<commit_message>
readjust some risk indicator for acct profiling
</commit_message>
<xml_diff>
--- a/Output/acct_profiling/account_profiling_summary.xlsx
+++ b/Output/acct_profiling/account_profiling_summary.xlsx
@@ -1594,7 +1594,7 @@
         <v>0.48</v>
       </c>
       <c r="AQ6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR6" t="b">
         <v>1</v>
@@ -1776,7 +1776,7 @@
         <v>0</v>
       </c>
       <c r="AQ7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR7" t="b">
         <v>1</v>
@@ -1972,7 +1972,7 @@
         <v>0.87</v>
       </c>
       <c r="AQ8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR8" t="b">
         <v>1</v>
@@ -2156,7 +2156,7 @@
         <v>0</v>
       </c>
       <c r="AQ9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR9" t="b">
         <v>1</v>
@@ -2348,7 +2348,7 @@
         <v>0.85</v>
       </c>
       <c r="AQ10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR10" t="b">
         <v>1</v>
@@ -2540,7 +2540,7 @@
         <v>1.39</v>
       </c>
       <c r="AQ11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR11" t="b">
         <v>1</v>
@@ -2724,7 +2724,7 @@
         <v>0</v>
       </c>
       <c r="AQ12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR12" t="b">
         <v>1</v>
@@ -2908,7 +2908,7 @@
         <v>0</v>
       </c>
       <c r="AQ13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR13" t="b">
         <v>1</v>
@@ -3086,7 +3086,7 @@
         <v>0</v>
       </c>
       <c r="AQ14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR14" t="b">
         <v>1</v>
@@ -3270,7 +3270,7 @@
         <v>0</v>
       </c>
       <c r="AQ15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR15" t="b">
         <v>1</v>
@@ -3462,7 +3462,7 @@
         <v>1.72</v>
       </c>
       <c r="AQ16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR16" t="b">
         <v>1</v>
@@ -3646,7 +3646,7 @@
         <v>0</v>
       </c>
       <c r="AQ17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR17" t="b">
         <v>1</v>
@@ -3793,7 +3793,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3821,27 +3821,27 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1st Login HCM vs Order Can Tho</t>
+          <t>Missing Email</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>100</v>
+        <v>93.75</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Missing Email</t>
+          <t>Account Age &lt; 90 Days</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>93.75</v>
+        <v>87.5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Account Age &lt; 90 Days</t>
+          <t>Extreme High Freq (&lt;30s Lag)</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -3851,17 +3851,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Extreme High Freq (&lt;30s Lag)</t>
+          <t>Incomplete Profile Name</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>87.5</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Pre-Reg Order Anomaly</t>
+          <t>WEB Access Channel</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -3871,50 +3871,20 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Incomplete Profile Name</t>
+          <t>Zero Order Completion</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>75</v>
+        <v>62.5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>WEB Access Channel</t>
+          <t>Shared Device ID</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Zero Order Completion</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>62.5</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Corporate Account Flag</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>18.75</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Shared Device ID (Bot Farm)</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
         <v>18.75</v>
       </c>
     </row>

</xml_diff>